<commit_message>
Adding a wind process and demand to base
</commit_message>
<xml_diff>
--- a/VT_EE_DemElc_V01.xlsx
+++ b/VT_EE_DemElc_V01.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showObjects="placeholders" codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\VEDA_Models\PhD_Kristopher\EE-TIMES-New\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D704D821-22B0-4E79-A064-E2A2EEB234BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4376B573-4F34-4E5A-A4A0-C48519EE7D95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="38640" windowHeight="15720" tabRatio="901" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" tabRatio="901" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DemTechs_TPS" sheetId="136" r:id="rId1"/>
@@ -346,7 +346,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R9" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0300-000006000000}">
+    <comment ref="S9" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0300-000006000000}">
       <text>
         <r>
           <rPr>
@@ -439,7 +439,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S9" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-000007000000}">
+    <comment ref="T9" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0300-000007000000}">
       <text>
         <r>
           <rPr>
@@ -464,7 +464,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T9" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0300-000008000000}">
+    <comment ref="U9" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0300-000008000000}">
       <text>
         <r>
           <rPr>
@@ -527,7 +527,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L10" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0300-000009000000}">
+    <comment ref="M10" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0300-000009000000}">
       <text>
         <r>
           <rPr>
@@ -775,7 +775,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="104">
   <si>
     <t>CommName</t>
   </si>
@@ -912,9 +912,6 @@
     <t>Description</t>
   </si>
   <si>
-    <t>PJ</t>
-  </si>
-  <si>
     <t>Default Unit</t>
   </si>
   <si>
@@ -984,9 +981,6 @@
     <t>Lifetime</t>
   </si>
   <si>
-    <t>Pja</t>
-  </si>
-  <si>
     <t>ELCC</t>
   </si>
   <si>
@@ -1081,18 +1075,29 @@
   </si>
   <si>
     <t>S04H06</t>
+  </si>
+  <si>
+    <t>TWh</t>
+  </si>
+  <si>
+    <t>GW</t>
+  </si>
+  <si>
+    <t>CAP2ACT</t>
+  </si>
+  <si>
+    <t>Capacity to Activity Factor</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="\Te\x\t"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="\Te\x\t"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1185,6 +1190,10 @@
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="10">
@@ -1289,7 +1298,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="17">
+  <cellStyleXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -1307,6 +1316,7 @@
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1334,7 +1344,6 @@
     </xf>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="6" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="1" fontId="3" fillId="8" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="4" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="8" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1363,27 +1372,28 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="3" fillId="8" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="9" borderId="0" xfId="17" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="17">
+  <cellStyles count="18">
     <cellStyle name="20% - Accent5" xfId="1" builtinId="46"/>
     <cellStyle name="Accent2" xfId="2" builtinId="33"/>
     <cellStyle name="Comma 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
@@ -1397,6 +1407,7 @@
     <cellStyle name="Normal 8" xfId="10" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
     <cellStyle name="Normal 9 2" xfId="11" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
     <cellStyle name="Normale_B2020" xfId="12" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
+    <cellStyle name="Percent" xfId="17" builtinId="5"/>
     <cellStyle name="Percent 2" xfId="13" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
     <cellStyle name="Percent 3" xfId="14" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
     <cellStyle name="Percent 4" xfId="15" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
@@ -2057,31 +2068,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="B1:T27"/>
-  <sheetFormatPr defaultRowHeight="12.3" x14ac:dyDescent="0.4"/>
+  <dimension ref="B1:U27"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
-    <col min="2" max="2" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.27734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="9.27734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="2.71875" customWidth="1"/>
-    <col min="12" max="12" width="12.71875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.1640625" customWidth="1"/>
-    <col min="14" max="14" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="42.5546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.71875" customWidth="1"/>
-    <col min="18" max="18" width="13.44140625" customWidth="1"/>
-    <col min="19" max="19" width="13.83203125" customWidth="1"/>
-    <col min="20" max="20" width="8.44140625" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.140625" customWidth="1"/>
+    <col min="14" max="14" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="42.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.7109375" customWidth="1"/>
+    <col min="18" max="18" width="13.42578125" customWidth="1"/>
+    <col min="19" max="19" width="13.85546875" customWidth="1"/>
+    <col min="20" max="20" width="8.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:20" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="2:21" ht="15" x14ac:dyDescent="0.25">
       <c r="B1" s="6" t="s">
         <v>43</v>
       </c>
@@ -2089,190 +2100,193 @@
         <v>44</v>
       </c>
       <c r="D1" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="H1" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E1" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="2" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="L2" s="26" t="s">
+    </row>
+    <row r="2" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="L2" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="M2" s="26"/>
-      <c r="N2" s="27"/>
-      <c r="O2" s="27"/>
-      <c r="P2" s="27"/>
-      <c r="Q2" s="27"/>
-      <c r="R2" s="27"/>
-      <c r="S2" s="27"/>
-      <c r="T2" s="27"/>
-    </row>
-    <row r="3" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="L3" s="28" t="s">
+      <c r="M2" s="25"/>
+      <c r="N2" s="26"/>
+      <c r="O2" s="26"/>
+      <c r="P2" s="26"/>
+      <c r="Q2" s="26"/>
+      <c r="R2" s="26"/>
+      <c r="S2" s="26"/>
+      <c r="T2" s="26"/>
+    </row>
+    <row r="3" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="L3" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="M3" s="29" t="s">
+      <c r="M3" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="N3" s="28" t="s">
+      <c r="N3" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="O3" s="28" t="s">
+      <c r="O3" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="P3" s="28" t="s">
+      <c r="P3" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="Q3" s="28" t="s">
+      <c r="Q3" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="R3" s="28" t="s">
+      <c r="R3" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="S3" s="28" t="s">
+      <c r="S3" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="T3" s="28" t="s">
+      <c r="T3" s="27" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="2:20" ht="21" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="L4" s="30" t="s">
+    <row r="4" spans="2:21" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="L4" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="M4" s="30" t="s">
+      <c r="M4" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="N4" s="30" t="s">
+      <c r="N4" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="O4" s="30" t="s">
+      <c r="O4" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="P4" s="30" t="s">
+      <c r="P4" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="Q4" s="30" t="s">
+      <c r="Q4" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="R4" s="30" t="s">
+      <c r="R4" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="S4" s="30" t="s">
+      <c r="S4" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="T4" s="30" t="s">
+      <c r="T4" s="29" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="2:20" ht="15.6" x14ac:dyDescent="0.6">
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
+    <row r="5" spans="2:21" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
       <c r="L5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="N5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="O5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="P5" t="s">
-        <v>45</v>
-      </c>
-      <c r="Q5" s="27"/>
-      <c r="R5" s="27"/>
-      <c r="S5" s="27"/>
-      <c r="T5" s="27"/>
-    </row>
-    <row r="8" spans="2:20" x14ac:dyDescent="0.4">
+        <v>100</v>
+      </c>
+      <c r="Q5" s="26"/>
+      <c r="R5" s="26"/>
+      <c r="S5" s="26"/>
+      <c r="T5" s="26"/>
+    </row>
+    <row r="8" spans="2:21" x14ac:dyDescent="0.2">
       <c r="D8" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="H8" s="4"/>
-      <c r="I8" s="15"/>
-      <c r="J8" s="16"/>
-      <c r="L8" s="26" t="s">
+      <c r="I8" s="14"/>
+      <c r="J8" s="15"/>
+      <c r="L8" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="M8" s="26"/>
-      <c r="N8" s="31"/>
-      <c r="O8" s="31"/>
-      <c r="P8" s="31"/>
-      <c r="Q8" s="31"/>
-      <c r="R8" s="31"/>
-      <c r="S8" s="31"/>
-      <c r="T8" s="31"/>
-    </row>
-    <row r="9" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B9" s="18" t="s">
+      <c r="M8" s="25"/>
+      <c r="N8" s="30"/>
+      <c r="O8" s="30"/>
+      <c r="P8" s="30"/>
+      <c r="Q8" s="30"/>
+      <c r="R8" s="30"/>
+      <c r="S8" s="30"/>
+      <c r="T8" s="30"/>
+    </row>
+    <row r="9" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B9" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="23" t="s">
+      <c r="E9" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="G9" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="H9" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="H9" s="18" t="s">
+      <c r="I9" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="I9" s="18" t="s">
+      <c r="J9" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="K9" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="J9" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="L9" s="28" t="s">
+      <c r="M9" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="M9" s="29" t="s">
+      <c r="N9" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="N9" s="28" t="s">
+      <c r="O9" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="O9" s="28" t="s">
+      <c r="P9" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="P9" s="28" t="s">
+      <c r="Q9" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="Q9" s="28" t="s">
+      <c r="R9" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="R9" s="28" t="s">
+      <c r="S9" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="S9" s="28" t="s">
+      <c r="T9" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="T9" s="28" t="s">
+      <c r="U9" s="27" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="2:20" ht="21" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:21" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B10" s="9" t="s">
         <v>38</v>
       </c>
@@ -2283,54 +2297,57 @@
         <v>33</v>
       </c>
       <c r="E10" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="F10" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="G10" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="G10" s="22" t="s">
+      <c r="H10" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="I10" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="I10" s="9" t="s">
-        <v>65</v>
-      </c>
       <c r="J10" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="L10" s="30" t="s">
+        <v>103</v>
+      </c>
+      <c r="K10" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="M10" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="M10" s="30" t="s">
+      <c r="N10" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="N10" s="30" t="s">
+      <c r="O10" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="O10" s="30" t="s">
+      <c r="P10" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="P10" s="30" t="s">
+      <c r="Q10" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="Q10" s="30" t="s">
+      <c r="R10" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="R10" s="30" t="s">
+      <c r="S10" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="S10" s="30" t="s">
+      <c r="T10" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="T10" s="30" t="s">
+      <c r="U10" s="29" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="2:20" ht="12.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:21" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B11" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C11" s="8"/>
       <c r="D11" s="8"/>
@@ -2339,7 +2356,7 @@
         <v>a</v>
       </c>
       <c r="F11" s="7"/>
-      <c r="G11" s="19"/>
+      <c r="G11" s="18"/>
       <c r="H11" s="7" t="str">
         <f>$F$2&amp;"/"&amp;$E$2</f>
         <v>/</v>
@@ -2348,99 +2365,96 @@
         <f>$F$2&amp;"/"&amp;$E$2&amp;"a"</f>
         <v>/a</v>
       </c>
-      <c r="J11" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="L11" s="30" t="s">
-        <v>49</v>
-      </c>
-      <c r="M11" s="30"/>
-      <c r="N11" s="30"/>
-      <c r="O11" s="30"/>
-      <c r="P11" s="30"/>
-      <c r="Q11" s="30"/>
-      <c r="R11" s="30"/>
-      <c r="S11" s="30"/>
-      <c r="T11" s="30"/>
-    </row>
-    <row r="12" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B12" s="31" t="str">
-        <f>N12</f>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="M11" s="29" t="s">
+        <v>48</v>
+      </c>
+      <c r="N11" s="29"/>
+      <c r="O11" s="29"/>
+      <c r="P11" s="29"/>
+      <c r="Q11" s="29"/>
+      <c r="R11" s="29"/>
+      <c r="S11" s="29"/>
+      <c r="T11" s="29"/>
+      <c r="U11" s="29"/>
+    </row>
+    <row r="12" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B12" s="30" t="str">
+        <f>O12</f>
         <v>DTECHELC</v>
       </c>
       <c r="C12" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D12" t="str">
         <f>N5</f>
         <v>DEMELC</v>
       </c>
-      <c r="F12" s="20">
+      <c r="F12" s="19">
         <v>1</v>
       </c>
-      <c r="G12" s="20">
-        <v>0.95</v>
-      </c>
-      <c r="H12" s="12">
-        <v>10</v>
-      </c>
-      <c r="I12" s="20">
-        <f>H12*0.02</f>
-        <v>0.2</v>
-      </c>
-      <c r="J12" s="12">
+      <c r="G12" s="19"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="19"/>
+      <c r="J12" s="19">
+        <v>8.76</v>
+      </c>
+      <c r="K12" s="12">
         <v>20</v>
       </c>
-      <c r="L12" s="27" t="s">
-        <v>67</v>
-      </c>
-      <c r="M12" s="31"/>
-      <c r="N12" s="31" t="s">
-        <v>76</v>
-      </c>
-      <c r="O12" s="31" t="s">
-        <v>77</v>
-      </c>
-      <c r="P12" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="Q12" s="34" t="s">
-        <v>69</v>
-      </c>
-      <c r="R12" s="31"/>
-      <c r="S12" s="31"/>
-      <c r="T12" s="31"/>
-    </row>
-    <row r="13" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="M12" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="N12" s="30"/>
+      <c r="O12" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="P12" s="30" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q12" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="R12" s="32" t="s">
+        <v>101</v>
+      </c>
+      <c r="S12" s="30"/>
+      <c r="T12" s="30"/>
+      <c r="U12" s="30"/>
+    </row>
+    <row r="13" spans="2:21" x14ac:dyDescent="0.2">
       <c r="E13" s="5"/>
-      <c r="F13" s="21"/>
-      <c r="G13" s="21"/>
-      <c r="I13" s="21"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="I13" s="20"/>
       <c r="O13" s="10"/>
     </row>
-    <row r="14" spans="2:20" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:21" x14ac:dyDescent="0.2">
       <c r="E14" s="5"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
-      <c r="I14" s="21"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="I14" s="20"/>
       <c r="O14" s="10"/>
     </row>
-    <row r="17" spans="9:11" x14ac:dyDescent="0.4">
-      <c r="I17" s="17"/>
-    </row>
-    <row r="18" spans="9:11" x14ac:dyDescent="0.4">
-      <c r="I18" s="17"/>
-    </row>
-    <row r="24" spans="9:11" x14ac:dyDescent="0.4">
+    <row r="17" spans="9:11" x14ac:dyDescent="0.2">
+      <c r="I17" s="16"/>
+    </row>
+    <row r="18" spans="9:11" x14ac:dyDescent="0.2">
+      <c r="I18" s="16"/>
+    </row>
+    <row r="24" spans="9:11" x14ac:dyDescent="0.2">
       <c r="K24" s="1"/>
     </row>
-    <row r="25" spans="9:11" x14ac:dyDescent="0.4">
+    <row r="25" spans="9:11" x14ac:dyDescent="0.2">
       <c r="K25" s="1"/>
     </row>
-    <row r="26" spans="9:11" x14ac:dyDescent="0.4">
+    <row r="26" spans="9:11" x14ac:dyDescent="0.2">
       <c r="K26" s="1"/>
     </row>
-    <row r="27" spans="9:11" x14ac:dyDescent="0.4">
+    <row r="27" spans="9:11" x14ac:dyDescent="0.2">
       <c r="K27" s="1"/>
     </row>
   </sheetData>
@@ -2452,20 +2466,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="B3:L30"/>
-  <sheetFormatPr defaultRowHeight="12.3" x14ac:dyDescent="0.4"/>
+  <dimension ref="B3:M34"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.27734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.27734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="12.44140625" customWidth="1"/>
-    <col min="10" max="10" width="7.27734375" customWidth="1"/>
-    <col min="11" max="11" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="12.42578125" customWidth="1"/>
+    <col min="10" max="10" width="7.28515625" customWidth="1"/>
+    <col min="11" max="11" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:10" x14ac:dyDescent="0.2">
       <c r="C3" s="3" t="s">
         <v>13</v>
       </c>
@@ -2475,9 +2489,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B4" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>0</v>
@@ -2485,51 +2499,51 @@
       <c r="D4" s="2">
         <v>2025</v>
       </c>
-      <c r="F4" s="24"/>
-      <c r="G4" s="32" t="s">
-        <v>74</v>
-      </c>
-      <c r="H4" s="24" t="s">
+      <c r="F4" s="23"/>
+      <c r="G4" s="31" t="s">
+        <v>72</v>
+      </c>
+      <c r="H4" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="I4" s="24" t="s">
-        <v>73</v>
-      </c>
-      <c r="J4" s="24">
+      <c r="I4" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="J4" s="23">
         <v>2025</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="20.7" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:10" ht="22.5" x14ac:dyDescent="0.2">
       <c r="B5" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>49</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>50</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25" t="s">
-        <v>49</v>
-      </c>
-      <c r="I5" s="25"/>
-      <c r="J5" s="25"/>
-    </row>
-    <row r="6" spans="2:12" ht="12.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="F5" s="24"/>
+      <c r="G5" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
+    </row>
+    <row r="6" spans="2:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B6" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25" t="s">
-        <v>49</v>
-      </c>
-      <c r="I6" s="25"/>
-      <c r="J6" s="25"/>
-    </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="F6" s="24"/>
+      <c r="G6" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="I6" s="24"/>
+      <c r="J6" s="24"/>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>34</v>
       </c>
@@ -2537,327 +2551,377 @@
         <f>DemTechs_TPS!N5</f>
         <v>DEMELC</v>
       </c>
-      <c r="D7" s="13"/>
+      <c r="D7" s="34">
+        <v>7.94</v>
+      </c>
       <c r="G7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H7" t="str">
         <f>$C$7</f>
         <v>DEMELC</v>
       </c>
       <c r="I7" t="s">
-        <v>78</v>
-      </c>
-      <c r="J7" s="35"/>
-      <c r="L7" s="33"/>
-    </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.4">
+        <v>76</v>
+      </c>
+      <c r="J7" s="33">
+        <v>3.9907549910668097E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.2">
       <c r="E8" s="5"/>
       <c r="G8" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H8" t="str">
         <f t="shared" ref="H8:H30" si="0">$C$7</f>
         <v>DEMELC</v>
       </c>
       <c r="I8" t="s">
-        <v>79</v>
-      </c>
-      <c r="J8" s="35"/>
-      <c r="L8" s="33"/>
-    </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.4">
+        <v>77</v>
+      </c>
+      <c r="J8" s="33">
+        <v>4.2568441071658941E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.2">
       <c r="G9" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H9" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I9" t="s">
-        <v>80</v>
-      </c>
-      <c r="J9" s="35"/>
-      <c r="L9" s="33"/>
-    </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.4">
+        <v>78</v>
+      </c>
+      <c r="J9" s="33">
+        <v>4.9357090706698532E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.2">
       <c r="E10" s="11"/>
       <c r="G10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H10" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I10" t="s">
-        <v>81</v>
-      </c>
-      <c r="J10" s="35"/>
-      <c r="L10" s="33"/>
-    </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.4">
+        <v>79</v>
+      </c>
+      <c r="J10" s="33">
+        <v>4.6935749761719207E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.2">
       <c r="E11" s="5"/>
       <c r="G11" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H11" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I11" t="s">
-        <v>82</v>
-      </c>
-      <c r="J11" s="35"/>
-      <c r="L11" s="33"/>
-    </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.4">
+        <v>80</v>
+      </c>
+      <c r="J11" s="33">
+        <v>5.0324370403048241E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.2">
       <c r="G12" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H12" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I12" t="s">
-        <v>83</v>
-      </c>
-      <c r="J12" s="35"/>
-      <c r="L12" s="33"/>
-    </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.4">
+        <v>81</v>
+      </c>
+      <c r="J12" s="33">
+        <v>4.644570688133022E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.2">
       <c r="E13" s="5"/>
       <c r="G13" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H13" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I13" t="s">
-        <v>84</v>
-      </c>
-      <c r="J13" s="36"/>
-    </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.4">
+        <v>82</v>
+      </c>
+      <c r="J13" s="35">
+        <v>3.198760977379362E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.2">
       <c r="G14" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H14" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I14" t="s">
-        <v>85</v>
-      </c>
-      <c r="J14" s="36"/>
-    </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.4">
+        <v>83</v>
+      </c>
+      <c r="J14" s="35">
+        <v>3.450628688202826E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.2">
       <c r="G15" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H15" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I15" t="s">
-        <v>86</v>
-      </c>
-      <c r="J15" s="36"/>
-    </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.4">
+        <v>84</v>
+      </c>
+      <c r="J15" s="35">
+        <v>4.1710976210981882E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10" x14ac:dyDescent="0.2">
       <c r="G16" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H16" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I16" t="s">
-        <v>87</v>
-      </c>
-      <c r="J16" s="36"/>
-    </row>
-    <row r="17" spans="7:10" x14ac:dyDescent="0.4">
+        <v>85</v>
+      </c>
+      <c r="J16" s="35">
+        <v>4.110700091078253E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G17" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H17" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I17" t="s">
-        <v>88</v>
-      </c>
-      <c r="J17" s="36"/>
-    </row>
-    <row r="18" spans="7:10" x14ac:dyDescent="0.4">
+        <v>86</v>
+      </c>
+      <c r="J17" s="35">
+        <v>3.8350662386599552E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G18" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H18" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I18" t="s">
-        <v>89</v>
-      </c>
-      <c r="J18" s="36"/>
-    </row>
-    <row r="19" spans="7:10" x14ac:dyDescent="0.4">
+        <v>87</v>
+      </c>
+      <c r="J18" s="35">
+        <v>3.7409762931132108E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G19" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H19" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I19" t="s">
-        <v>90</v>
-      </c>
-      <c r="J19" s="36"/>
-    </row>
-    <row r="20" spans="7:10" x14ac:dyDescent="0.4">
+        <v>88</v>
+      </c>
+      <c r="J19" s="35">
+        <v>3.1132436657193206E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G20" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H20" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I20" t="s">
-        <v>91</v>
-      </c>
-      <c r="J20" s="36"/>
-    </row>
-    <row r="21" spans="7:10" x14ac:dyDescent="0.4">
+        <v>89</v>
+      </c>
+      <c r="J20" s="35">
+        <v>3.3429633070020642E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G21" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H21" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I21" t="s">
-        <v>92</v>
-      </c>
-      <c r="J21" s="36"/>
-    </row>
-    <row r="22" spans="7:10" x14ac:dyDescent="0.4">
+        <v>90</v>
+      </c>
+      <c r="J21" s="35">
+        <v>4.2259483749326171E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G22" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H22" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I22" t="s">
-        <v>93</v>
-      </c>
-      <c r="J22" s="36"/>
-    </row>
-    <row r="23" spans="7:10" x14ac:dyDescent="0.4">
+        <v>91</v>
+      </c>
+      <c r="J22" s="35">
+        <v>4.1634467216423117E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G23" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H23" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I23" t="s">
-        <v>94</v>
-      </c>
-      <c r="J23" s="36"/>
-    </row>
-    <row r="24" spans="7:10" x14ac:dyDescent="0.4">
+        <v>92</v>
+      </c>
+      <c r="J23" s="35">
+        <v>3.9259389280991014E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G24" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H24" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I24" t="s">
-        <v>95</v>
-      </c>
-      <c r="J24" s="36"/>
-    </row>
-    <row r="25" spans="7:10" x14ac:dyDescent="0.4">
+        <v>93</v>
+      </c>
+      <c r="J24" s="35">
+        <v>3.742541478765557E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G25" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H25" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I25" t="s">
-        <v>96</v>
-      </c>
-      <c r="J25" s="36"/>
-    </row>
-    <row r="26" spans="7:10" x14ac:dyDescent="0.4">
+        <v>94</v>
+      </c>
+      <c r="J25" s="35">
+        <v>3.8818644082250733E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G26" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H26" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I26" t="s">
-        <v>97</v>
-      </c>
-      <c r="J26" s="36"/>
-    </row>
-    <row r="27" spans="7:10" x14ac:dyDescent="0.4">
+        <v>95</v>
+      </c>
+      <c r="J26" s="35">
+        <v>4.101069729156176E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G27" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H27" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I27" t="s">
-        <v>98</v>
-      </c>
-      <c r="J27" s="36"/>
-    </row>
-    <row r="28" spans="7:10" x14ac:dyDescent="0.4">
+        <v>96</v>
+      </c>
+      <c r="J27" s="35">
+        <v>4.9652911424591967E-2</v>
+      </c>
+    </row>
+    <row r="28" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G28" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H28" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I28" t="s">
-        <v>99</v>
-      </c>
-      <c r="J28" s="36"/>
-    </row>
-    <row r="29" spans="7:10" x14ac:dyDescent="0.4">
+        <v>97</v>
+      </c>
+      <c r="J28" s="35">
+        <v>4.9211095905815884E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G29" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H29" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I29" t="s">
-        <v>100</v>
-      </c>
-      <c r="J29" s="36"/>
-    </row>
-    <row r="30" spans="7:10" x14ac:dyDescent="0.4">
+        <v>98</v>
+      </c>
+      <c r="J29" s="35">
+        <v>5.0243422728341029E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G30" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H30" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I30" t="s">
-        <v>101</v>
-      </c>
-      <c r="J30" s="36"/>
+        <v>99</v>
+      </c>
+      <c r="J30" s="35">
+        <v>4.5311195975387637E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="13:13" x14ac:dyDescent="0.2">
+      <c r="M34" s="36">
+        <f>SUM(J7:J30)</f>
+        <v>1.0000000000000002</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Error fix from previous commit
</commit_message>
<xml_diff>
--- a/VT_EE_DemElc_V01.xlsx
+++ b/VT_EE_DemElc_V01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4376B573-4F34-4E5A-A4A0-C48519EE7D95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{181D18BE-ABEC-4DD4-A801-122345DF7C38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" tabRatio="901" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" tabRatio="901" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DemTechs_TPS" sheetId="136" r:id="rId1"/>
@@ -2082,7 +2082,7 @@
     <col min="10" max="10" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.140625" customWidth="1"/>
+    <col min="13" max="13" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="42.5703125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="7.42578125" bestFit="1" customWidth="1"/>
@@ -2215,10 +2215,9 @@
       <c r="H8" s="4"/>
       <c r="I8" s="14"/>
       <c r="J8" s="15"/>
-      <c r="L8" s="25" t="s">
+      <c r="M8" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="M8" s="25"/>
       <c r="N8" s="30"/>
       <c r="O8" s="30"/>
       <c r="P8" s="30"/>

</xml_diff>

<commit_message>
changing elcc to elc
</commit_message>
<xml_diff>
--- a/VT_EE_DemElc_V01.xlsx
+++ b/VT_EE_DemElc_V01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{181D18BE-ABEC-4DD4-A801-122345DF7C38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB903054-CC9E-4A2B-953D-BCE23A6E7A94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" tabRatio="901" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" tabRatio="901" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DemTechs_TPS" sheetId="136" r:id="rId1"/>
@@ -981,9 +981,6 @@
     <t>Lifetime</t>
   </si>
   <si>
-    <t>ELCC</t>
-  </si>
-  <si>
     <t>Demand of electricity in all sectors</t>
   </si>
   <si>
@@ -1087,6 +1084,9 @@
   </si>
   <si>
     <t>Capacity to Activity Factor</t>
+  </si>
+  <si>
+    <t>ELC</t>
   </si>
 </sst>
 </file>
@@ -2193,13 +2193,13 @@
         <v>50</v>
       </c>
       <c r="N5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="O5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="P5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q5" s="26"/>
       <c r="R5" s="26"/>
@@ -2252,7 +2252,7 @@
         <v>58</v>
       </c>
       <c r="J9" s="17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="K9" s="22" t="s">
         <v>59</v>
@@ -2311,7 +2311,7 @@
         <v>64</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K10" s="9" t="s">
         <v>67</v>
@@ -2386,7 +2386,7 @@
         <v>DTECHELC</v>
       </c>
       <c r="C12" t="s">
-        <v>68</v>
+        <v>103</v>
       </c>
       <c r="D12" t="str">
         <f>N5</f>
@@ -2409,16 +2409,16 @@
       </c>
       <c r="N12" s="30"/>
       <c r="O12" s="30" t="s">
+        <v>73</v>
+      </c>
+      <c r="P12" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="P12" s="30" t="s">
-        <v>75</v>
-      </c>
       <c r="Q12" s="32" t="s">
+        <v>99</v>
+      </c>
+      <c r="R12" s="32" t="s">
         <v>100</v>
-      </c>
-      <c r="R12" s="32" t="s">
-        <v>101</v>
       </c>
       <c r="S12" s="30"/>
       <c r="T12" s="30"/>
@@ -2500,13 +2500,13 @@
       </c>
       <c r="F4" s="23"/>
       <c r="G4" s="31" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H4" s="23" t="s">
         <v>0</v>
       </c>
       <c r="I4" s="23" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J4" s="23">
         <v>2025</v>
@@ -2554,14 +2554,14 @@
         <v>7.94</v>
       </c>
       <c r="G7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H7" t="str">
         <f>$C$7</f>
         <v>DEMELC</v>
       </c>
       <c r="I7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J7" s="33">
         <v>3.9907549910668097E-2</v>
@@ -2570,14 +2570,14 @@
     <row r="8" spans="2:10" x14ac:dyDescent="0.2">
       <c r="E8" s="5"/>
       <c r="G8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H8" t="str">
         <f t="shared" ref="H8:H30" si="0">$C$7</f>
         <v>DEMELC</v>
       </c>
       <c r="I8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J8" s="33">
         <v>4.2568441071658941E-2</v>
@@ -2585,14 +2585,14 @@
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.2">
       <c r="G9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H9" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J9" s="33">
         <v>4.9357090706698532E-2</v>
@@ -2601,14 +2601,14 @@
     <row r="10" spans="2:10" x14ac:dyDescent="0.2">
       <c r="E10" s="11"/>
       <c r="G10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H10" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J10" s="33">
         <v>4.6935749761719207E-2</v>
@@ -2617,14 +2617,14 @@
     <row r="11" spans="2:10" x14ac:dyDescent="0.2">
       <c r="E11" s="5"/>
       <c r="G11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H11" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J11" s="33">
         <v>5.0324370403048241E-2</v>
@@ -2632,14 +2632,14 @@
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.2">
       <c r="G12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H12" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J12" s="33">
         <v>4.644570688133022E-2</v>
@@ -2648,14 +2648,14 @@
     <row r="13" spans="2:10" x14ac:dyDescent="0.2">
       <c r="E13" s="5"/>
       <c r="G13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H13" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J13" s="35">
         <v>3.198760977379362E-2</v>
@@ -2663,14 +2663,14 @@
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.2">
       <c r="G14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H14" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J14" s="35">
         <v>3.450628688202826E-2</v>
@@ -2678,14 +2678,14 @@
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.2">
       <c r="G15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H15" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I15" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J15" s="35">
         <v>4.1710976210981882E-2</v>
@@ -2693,14 +2693,14 @@
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.2">
       <c r="G16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H16" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I16" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J16" s="35">
         <v>4.110700091078253E-2</v>
@@ -2708,14 +2708,14 @@
     </row>
     <row r="17" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H17" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I17" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J17" s="35">
         <v>3.8350662386599552E-2</v>
@@ -2723,14 +2723,14 @@
     </row>
     <row r="18" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H18" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="J18" s="35">
         <v>3.7409762931132108E-2</v>
@@ -2738,14 +2738,14 @@
     </row>
     <row r="19" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G19" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H19" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I19" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J19" s="35">
         <v>3.1132436657193206E-2</v>
@@ -2753,14 +2753,14 @@
     </row>
     <row r="20" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G20" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H20" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I20" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J20" s="35">
         <v>3.3429633070020642E-2</v>
@@ -2768,14 +2768,14 @@
     </row>
     <row r="21" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H21" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J21" s="35">
         <v>4.2259483749326171E-2</v>
@@ -2783,14 +2783,14 @@
     </row>
     <row r="22" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H22" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I22" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="J22" s="35">
         <v>4.1634467216423117E-2</v>
@@ -2798,14 +2798,14 @@
     </row>
     <row r="23" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H23" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I23" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J23" s="35">
         <v>3.9259389280991014E-2</v>
@@ -2813,14 +2813,14 @@
     </row>
     <row r="24" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G24" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H24" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I24" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J24" s="35">
         <v>3.742541478765557E-2</v>
@@ -2828,14 +2828,14 @@
     </row>
     <row r="25" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G25" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H25" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I25" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="J25" s="35">
         <v>3.8818644082250733E-2</v>
@@ -2843,14 +2843,14 @@
     </row>
     <row r="26" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G26" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H26" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I26" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="J26" s="35">
         <v>4.101069729156176E-2</v>
@@ -2858,14 +2858,14 @@
     </row>
     <row r="27" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G27" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H27" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I27" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J27" s="35">
         <v>4.9652911424591967E-2</v>
@@ -2873,14 +2873,14 @@
     </row>
     <row r="28" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G28" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H28" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I28" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J28" s="35">
         <v>4.9211095905815884E-2</v>
@@ -2888,14 +2888,14 @@
     </row>
     <row r="29" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G29" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H29" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I29" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J29" s="35">
         <v>5.0243422728341029E-2</v>
@@ -2903,14 +2903,14 @@
     </row>
     <row r="30" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G30" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H30" t="str">
         <f t="shared" si="0"/>
         <v>DEMELC</v>
       </c>
       <c r="I30" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J30" s="35">
         <v>4.5311195975387637E-2</v>

</xml_diff>

<commit_message>
Adding demand until 2050
</commit_message>
<xml_diff>
--- a/VT_EE_DemElc_V01.xlsx
+++ b/VT_EE_DemElc_V01.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB903054-CC9E-4A2B-953D-BCE23A6E7A94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71B18899-2C20-4EE0-8607-4A553D0D7FAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" tabRatio="901" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="901" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DemTechs_TPS" sheetId="136" r:id="rId1"/>
     <sheet name="Demands" sheetId="134" r:id="rId2"/>
+    <sheet name="SUBELCDEMTechs" sheetId="137" r:id="rId3"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId3"/>
+    <externalReference r:id="rId4"/>
   </externalReferences>
   <definedNames>
     <definedName name="FID_1">[1]AGR_Fuels!$A$2</definedName>
@@ -774,8 +775,743 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Gary Goldstein</author>
+    <author>Amit Kanudia</author>
+    <author>Maurizio Gargiulo</author>
+  </authors>
+  <commentList>
+    <comment ref="S6" authorId="0" shapeId="0" xr:uid="{6427DCF2-07B1-4689-ACCA-860F12C1F7C7}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Csets declarations are inherited until the next one is encountered.
+Allowed Cset:
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>NRG</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> (Energy)
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>ENV</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> (Emission)
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>DEM</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> (Demand)
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>MAT</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> (Material)
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>FIN</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> (Financial)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="X6" authorId="1" shapeId="0" xr:uid="{FE3400CE-D96E-4FE5-BD07-EA12F99EE43A}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Amit Kanudia:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+LO for PRODUCTION &gt;= CONSUMPTION (Default)
+FX for PRODUCTION = CONSUMPTION
+UP for PRODUCTION &lt;= CONSUMPTION</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y6" authorId="2" shapeId="0" xr:uid="{8DC047D6-E89E-45E9-980A-DF49A30415F6}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Allowed CTSLvl</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+SEASON</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> (Seasonal level)</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+WEEKLY</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> (Weekly level)</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+DAYNITE</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> (day and night level)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Z6" authorId="2" shapeId="0" xr:uid="{B60F0A83-F9D6-44F4-B1B2-31F7707A69FA}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Allowed PeakTS</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+ANNUAL </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>(to generate Peak Equation for all the TimeSlices)</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+User TS </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>(to generate Peak Equation for a single TS)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AA6" authorId="2" shapeId="0" xr:uid="{2B498BEA-1081-4088-85A1-1BCBFF765E9E}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Allowed Ctype
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>ELC</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> (Electricity)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y16" authorId="2" shapeId="0" xr:uid="{262E7131-99F0-41E9-9025-290199AF294F}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Allowed TsLvl
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>ANNUAL</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> (Annual level)
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>SEASON</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> (Seasonal level)
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>WEEKLY</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> (Weekly level)
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>DAYNITE</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> (day and night level)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Z16" authorId="1" shapeId="0" xr:uid="{7BE56FCE-5393-4AA0-8D0C-593832235C8F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Amit Kanudia:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Needed only when one wants to override the VEDA default assignment
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AA16" authorId="2" shapeId="0" xr:uid="{9059D6CB-1B2E-4106-81ED-22FDFBB8148D}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Allowed Vintage</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+NO</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> (if empty by default mean </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>NO</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>)</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+YES</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="S17" authorId="2" shapeId="0" xr:uid="{B4863F54-CA2E-4E29-A684-C0AE0DB06B52}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Sets declarations are </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>inherited. 
+Allowed Process Sets</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+ELE </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>(Thermal Electric Power Plant)</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+CHP </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>(Combined Heat and Power)</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+STGTSS </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>(Pump Storage)</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+STGIPS</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> (Pump Storage IP)</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+PRE </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>(Genric Process/Technology)</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+DMD</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> (Demand Device)</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+IMP </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">(Import)
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>EXP</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> (Export)</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+MIN </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>(Mining Process)</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+RNW </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>(Renewable Technology)</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+HPL</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> (Heating Plant)</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="120">
   <si>
     <t>CommName</t>
   </si>
@@ -1087,6 +1823,54 @@
   </si>
   <si>
     <t>ELC</t>
+  </si>
+  <si>
+    <t>DEMELC_COM</t>
+  </si>
+  <si>
+    <t>DEMELC_RSD</t>
+  </si>
+  <si>
+    <t>DEMELC_IND</t>
+  </si>
+  <si>
+    <t>DEMELC_TRA</t>
+  </si>
+  <si>
+    <t>Demand of Electricity in Commodity Sector</t>
+  </si>
+  <si>
+    <t>Demand of Electricity in Residential Sector</t>
+  </si>
+  <si>
+    <t>Demand of Electricity in Industry Sector</t>
+  </si>
+  <si>
+    <t>Demand of Electricity in Transport Sector</t>
+  </si>
+  <si>
+    <t>DTECHELC_COM</t>
+  </si>
+  <si>
+    <t>DTECHELC_RSD</t>
+  </si>
+  <si>
+    <t>DTECHELC_IND</t>
+  </si>
+  <si>
+    <t>DTECHELC_TRA</t>
+  </si>
+  <si>
+    <t>Demand Technologies of Electricity in Commodity Sector</t>
+  </si>
+  <si>
+    <t>Demand Technologies of Electricity in Residential Sector</t>
+  </si>
+  <si>
+    <t>Demand Technologies of Electricity in Transport Sector</t>
+  </si>
+  <si>
+    <t>Demand Technologies of Electricity in Industry Sector</t>
   </si>
 </sst>
 </file>
@@ -1194,6 +1978,8 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <charset val="186"/>
     </font>
   </fonts>
   <fills count="10">
@@ -1318,7 +2104,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1392,6 +2178,8 @@
     <xf numFmtId="2" fontId="3" fillId="8" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="9" borderId="0" xfId="17" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="18">
     <cellStyle name="20% - Accent5" xfId="1" builtinId="46"/>
@@ -2925,4 +3713,450 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01C3AA15-8F5C-44DF-A6DB-8A081DD06603}">
+  <dimension ref="C5:AA22"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="49.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="3:27" x14ac:dyDescent="0.2">
+      <c r="S5" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="T5" s="25"/>
+      <c r="U5" s="26"/>
+      <c r="V5" s="26"/>
+      <c r="W5" s="26"/>
+      <c r="X5" s="26"/>
+      <c r="Y5" s="26"/>
+      <c r="Z5" s="26"/>
+      <c r="AA5" s="26"/>
+    </row>
+    <row r="6" spans="3:27" x14ac:dyDescent="0.2">
+      <c r="S6" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="T6" s="28" t="s">
+        <v>30</v>
+      </c>
+      <c r="U6" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="V6" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="W6" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="X6" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="Y6" s="27" t="s">
+        <v>9</v>
+      </c>
+      <c r="Z6" s="27" t="s">
+        <v>10</v>
+      </c>
+      <c r="AA6" s="27" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="3:27" ht="45.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="S7" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="T7" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="U7" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="V7" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="W7" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="X7" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y7" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="Z7" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="29" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="3:27" x14ac:dyDescent="0.2">
+      <c r="S8" t="s">
+        <v>50</v>
+      </c>
+      <c r="U8" s="37" t="s">
+        <v>104</v>
+      </c>
+      <c r="V8" s="37" t="s">
+        <v>108</v>
+      </c>
+      <c r="W8" t="s">
+        <v>99</v>
+      </c>
+      <c r="X8" s="26"/>
+      <c r="Y8" s="26"/>
+      <c r="Z8" s="26"/>
+      <c r="AA8" s="26"/>
+    </row>
+    <row r="9" spans="3:27" x14ac:dyDescent="0.2">
+      <c r="S9" t="s">
+        <v>50</v>
+      </c>
+      <c r="U9" s="37" t="s">
+        <v>105</v>
+      </c>
+      <c r="V9" s="37" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="10" spans="3:27" x14ac:dyDescent="0.2">
+      <c r="S10" t="s">
+        <v>50</v>
+      </c>
+      <c r="U10" s="37" t="s">
+        <v>106</v>
+      </c>
+      <c r="V10" s="37" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="11" spans="3:27" x14ac:dyDescent="0.2">
+      <c r="S11" t="s">
+        <v>50</v>
+      </c>
+      <c r="U11" s="37" t="s">
+        <v>107</v>
+      </c>
+      <c r="V11" s="37" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="15" spans="3:27" x14ac:dyDescent="0.2">
+      <c r="E15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="14"/>
+      <c r="K15" s="15"/>
+      <c r="S15" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="T15" s="30"/>
+      <c r="U15" s="30"/>
+      <c r="V15" s="30"/>
+      <c r="W15" s="30"/>
+      <c r="X15" s="30"/>
+      <c r="Y15" s="30"/>
+      <c r="Z15" s="30"/>
+    </row>
+    <row r="16" spans="3:27" x14ac:dyDescent="0.2">
+      <c r="C16" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="D16" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="F16" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="G16" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="H16" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="I16" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="J16" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="K16" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="L16" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="S16" s="27" t="s">
+        <v>11</v>
+      </c>
+      <c r="T16" s="28" t="s">
+        <v>30</v>
+      </c>
+      <c r="U16" s="27" t="s">
+        <v>1</v>
+      </c>
+      <c r="V16" s="27" t="s">
+        <v>2</v>
+      </c>
+      <c r="W16" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="X16" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="Y16" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z16" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="AA16" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="3:27" ht="45.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C17" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H17" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="I17" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="J17" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="K17" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="L17" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="S17" s="29" t="s">
+        <v>37</v>
+      </c>
+      <c r="T17" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="U17" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="V17" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="W17" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="X17" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="Y17" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z17" s="29" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA17" s="29" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="3:27" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C18" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="7" t="str">
+        <f>E10&amp;"a"</f>
+        <v>a</v>
+      </c>
+      <c r="G18" s="7"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="7" t="str">
+        <f>$F$2&amp;"/"&amp;$E$2</f>
+        <v>/</v>
+      </c>
+      <c r="J18" s="7" t="str">
+        <f>$F$2&amp;"/"&amp;$E$2&amp;"a"</f>
+        <v>/a</v>
+      </c>
+      <c r="K18" s="7"/>
+      <c r="L18" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="S18" s="29" t="s">
+        <v>48</v>
+      </c>
+      <c r="T18" s="29"/>
+      <c r="U18" s="29"/>
+      <c r="V18" s="29"/>
+      <c r="W18" s="29"/>
+      <c r="X18" s="29"/>
+      <c r="Y18" s="29"/>
+      <c r="Z18" s="29"/>
+      <c r="AA18" s="29"/>
+    </row>
+    <row r="19" spans="3:27" x14ac:dyDescent="0.2">
+      <c r="C19" s="30" t="str">
+        <f>U19</f>
+        <v>DTECHELC_COM</v>
+      </c>
+      <c r="D19" t="str">
+        <f>DemTechs_TPS!$D$12</f>
+        <v>DEMELC</v>
+      </c>
+      <c r="E19" t="str">
+        <f>U8</f>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="G19" s="19">
+        <v>1</v>
+      </c>
+      <c r="H19" s="19"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="19">
+        <v>8.76</v>
+      </c>
+      <c r="L19" s="12">
+        <v>20</v>
+      </c>
+      <c r="S19" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="T19" s="30"/>
+      <c r="U19" s="38" t="s">
+        <v>112</v>
+      </c>
+      <c r="V19" s="37" t="s">
+        <v>116</v>
+      </c>
+      <c r="W19" s="32" t="s">
+        <v>99</v>
+      </c>
+      <c r="X19" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="Y19" s="30"/>
+      <c r="Z19" s="30"/>
+      <c r="AA19" s="30"/>
+    </row>
+    <row r="20" spans="3:27" x14ac:dyDescent="0.2">
+      <c r="C20" s="30" t="str">
+        <f t="shared" ref="C20:C22" si="0">U20</f>
+        <v>DTECHELC_RSD</v>
+      </c>
+      <c r="D20" t="str">
+        <f>DemTechs_TPS!$D$12</f>
+        <v>DEMELC</v>
+      </c>
+      <c r="E20" t="str">
+        <f t="shared" ref="E20:E22" si="1">U9</f>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="K20" s="19">
+        <v>8.76</v>
+      </c>
+      <c r="L20" s="12">
+        <v>20</v>
+      </c>
+      <c r="S20" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="U20" s="38" t="s">
+        <v>113</v>
+      </c>
+      <c r="V20" s="37" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="21" spans="3:27" x14ac:dyDescent="0.2">
+      <c r="C21" s="30" t="str">
+        <f t="shared" si="0"/>
+        <v>DTECHELC_IND</v>
+      </c>
+      <c r="D21" t="str">
+        <f>DemTechs_TPS!$D$12</f>
+        <v>DEMELC</v>
+      </c>
+      <c r="E21" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="K21" s="19">
+        <v>8.76</v>
+      </c>
+      <c r="L21" s="12">
+        <v>20</v>
+      </c>
+      <c r="S21" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="U21" s="38" t="s">
+        <v>114</v>
+      </c>
+      <c r="V21" s="37" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="22" spans="3:27" x14ac:dyDescent="0.2">
+      <c r="C22" s="30" t="str">
+        <f t="shared" si="0"/>
+        <v>DTECHELC_TRA</v>
+      </c>
+      <c r="D22" t="str">
+        <f>DemTechs_TPS!$D$12</f>
+        <v>DEMELC</v>
+      </c>
+      <c r="E22" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="K22" s="19">
+        <v>8.76</v>
+      </c>
+      <c r="L22" s="12">
+        <v>20</v>
+      </c>
+      <c r="S22" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="U22" s="38" t="s">
+        <v>115</v>
+      </c>
+      <c r="V22" s="37" t="s">
+        <v>118</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
commenting out fractions from total demand process
</commit_message>
<xml_diff>
--- a/VT_EE_DemElc_V01.xlsx
+++ b/VT_EE_DemElc_V01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D10CE1E0-22B4-4022-A50B-98A7E288E969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88DB72BC-DADA-40C9-94B1-229B68B95B9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="901" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" tabRatio="901" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DemTechs_TPS" sheetId="136" r:id="rId1"/>
@@ -1512,7 +1512,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="121">
   <si>
     <t>CommName</t>
   </si>
@@ -1872,6 +1872,9 @@
   </si>
   <si>
     <t>Demand Technologies of Electricity in Industry Sector</t>
+  </si>
+  <si>
+    <t>FI_T</t>
   </si>
 </sst>
 </file>
@@ -3274,7 +3277,7 @@
       <c r="D3" s="3"/>
       <c r="E3" s="1"/>
       <c r="J3" s="4" t="s">
-        <v>13</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Adding commodity fractions to demand
</commit_message>
<xml_diff>
--- a/VT_EE_DemElc_V01.xlsx
+++ b/VT_EE_DemElc_V01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88DB72BC-DADA-40C9-94B1-229B68B95B9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{951FF87C-51C9-4F10-AC41-3430C0B6C67C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="901" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="901" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DemTechs_TPS" sheetId="136" r:id="rId1"/>
@@ -1512,7 +1512,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="121">
   <si>
     <t>CommName</t>
   </si>
@@ -3266,7 +3266,7 @@
     <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="9" width="12.42578125" customWidth="1"/>
-    <col min="10" max="10" width="7.28515625" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4201,19 +4201,22 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47AEE53C-6660-4C48-A401-B5292118C9D7}">
-  <dimension ref="B3:I10"/>
+  <dimension ref="B3:T40"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:20" x14ac:dyDescent="0.2">
       <c r="C3" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="3"/>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B4" s="2" t="s">
         <v>47</v>
       </c>
@@ -4239,7 +4242,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="5" spans="2:9" ht="22.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:20" ht="22.5" x14ac:dyDescent="0.2">
       <c r="B5" s="9" t="s">
         <v>48</v>
       </c>
@@ -4265,7 +4268,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="2:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:20" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B6" s="8" t="s">
         <v>51</v>
       </c>
@@ -4277,7 +4280,7 @@
       <c r="H6" s="8"/>
       <c r="I6" s="8"/>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>34</v>
       </c>
@@ -4304,7 +4307,7 @@
         <v>4.798</v>
       </c>
     </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>34</v>
       </c>
@@ -4331,7 +4334,7 @@
         <v>3.306</v>
       </c>
     </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
         <v>34</v>
       </c>
@@ -4358,7 +4361,7 @@
         <v>3.206</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>34</v>
       </c>
@@ -4383,6 +4386,1410 @@
       </c>
       <c r="I10">
         <v>3.2690000000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q13" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B14" s="31" t="s">
+        <v>71</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="D14" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="E14" s="23">
+        <v>2025</v>
+      </c>
+      <c r="G14" s="31" t="s">
+        <v>71</v>
+      </c>
+      <c r="H14" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="I14" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="J14" s="23">
+        <v>2025</v>
+      </c>
+      <c r="L14" s="31" t="s">
+        <v>71</v>
+      </c>
+      <c r="M14" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="N14" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="O14" s="23">
+        <v>2025</v>
+      </c>
+      <c r="Q14" s="31" t="s">
+        <v>71</v>
+      </c>
+      <c r="R14" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="S14" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="T14" s="23">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="15" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B15" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="24"/>
+      <c r="E15" s="24"/>
+      <c r="G15" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="I15" s="24"/>
+      <c r="J15" s="24"/>
+      <c r="L15" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="N15" s="24"/>
+      <c r="O15" s="24"/>
+      <c r="Q15" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="S15" s="24"/>
+      <c r="T15" s="24"/>
+    </row>
+    <row r="16" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B16" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="G16" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="I16" s="24"/>
+      <c r="J16" s="24"/>
+      <c r="L16" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="N16" s="24"/>
+      <c r="O16" s="24"/>
+      <c r="Q16" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="S16" s="24"/>
+      <c r="T16" s="24"/>
+    </row>
+    <row r="17" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B17" t="s">
+        <v>72</v>
+      </c>
+      <c r="C17" t="str">
+        <f>C7</f>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D17" t="s">
+        <v>75</v>
+      </c>
+      <c r="E17" s="33">
+        <v>3.9907549910668097E-2</v>
+      </c>
+      <c r="G17" t="s">
+        <v>72</v>
+      </c>
+      <c r="H17" t="str">
+        <f>C8</f>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I17" t="s">
+        <v>75</v>
+      </c>
+      <c r="J17" s="33">
+        <v>3.9907549910668097E-2</v>
+      </c>
+      <c r="L17" t="s">
+        <v>72</v>
+      </c>
+      <c r="M17" t="str">
+        <f>C9</f>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N17" t="s">
+        <v>75</v>
+      </c>
+      <c r="O17" s="33">
+        <v>3.9907549910668097E-2</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>72</v>
+      </c>
+      <c r="R17" t="str">
+        <f>C10</f>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S17" t="s">
+        <v>75</v>
+      </c>
+      <c r="T17" s="33">
+        <v>3.9907549910668097E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C18" t="str">
+        <f t="shared" ref="C18:C40" si="0">$C$7</f>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D18" t="s">
+        <v>76</v>
+      </c>
+      <c r="E18" s="33">
+        <v>4.2568441071658941E-2</v>
+      </c>
+      <c r="G18" t="s">
+        <v>72</v>
+      </c>
+      <c r="H18" t="str">
+        <f>$C$8</f>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I18" t="s">
+        <v>76</v>
+      </c>
+      <c r="J18" s="33">
+        <v>4.2568441071658941E-2</v>
+      </c>
+      <c r="L18" t="s">
+        <v>72</v>
+      </c>
+      <c r="M18" t="str">
+        <f>$C$9</f>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N18" t="s">
+        <v>76</v>
+      </c>
+      <c r="O18" s="33">
+        <v>4.2568441071658941E-2</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>72</v>
+      </c>
+      <c r="R18" t="str">
+        <f>$C$10</f>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S18" t="s">
+        <v>76</v>
+      </c>
+      <c r="T18" s="33">
+        <v>4.2568441071658941E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>72</v>
+      </c>
+      <c r="C19" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D19" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19" s="33">
+        <v>4.9357090706698532E-2</v>
+      </c>
+      <c r="G19" t="s">
+        <v>72</v>
+      </c>
+      <c r="H19" t="str">
+        <f t="shared" ref="H19:H40" si="1">$C$8</f>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I19" t="s">
+        <v>77</v>
+      </c>
+      <c r="J19" s="33">
+        <v>4.9357090706698532E-2</v>
+      </c>
+      <c r="L19" t="s">
+        <v>72</v>
+      </c>
+      <c r="M19" t="str">
+        <f t="shared" ref="M19:M40" si="2">$C$9</f>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N19" t="s">
+        <v>77</v>
+      </c>
+      <c r="O19" s="33">
+        <v>4.9357090706698532E-2</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>72</v>
+      </c>
+      <c r="R19" t="str">
+        <f t="shared" ref="R19:R40" si="3">$C$10</f>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S19" t="s">
+        <v>77</v>
+      </c>
+      <c r="T19" s="33">
+        <v>4.9357090706698532E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
+        <v>72</v>
+      </c>
+      <c r="C20" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D20" t="s">
+        <v>78</v>
+      </c>
+      <c r="E20" s="33">
+        <v>4.6935749761719207E-2</v>
+      </c>
+      <c r="G20" t="s">
+        <v>72</v>
+      </c>
+      <c r="H20" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I20" t="s">
+        <v>78</v>
+      </c>
+      <c r="J20" s="33">
+        <v>4.6935749761719207E-2</v>
+      </c>
+      <c r="L20" t="s">
+        <v>72</v>
+      </c>
+      <c r="M20" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N20" t="s">
+        <v>78</v>
+      </c>
+      <c r="O20" s="33">
+        <v>4.6935749761719207E-2</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>72</v>
+      </c>
+      <c r="R20" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S20" t="s">
+        <v>78</v>
+      </c>
+      <c r="T20" s="33">
+        <v>4.6935749761719207E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B21" t="s">
+        <v>72</v>
+      </c>
+      <c r="C21" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D21" t="s">
+        <v>79</v>
+      </c>
+      <c r="E21" s="33">
+        <v>5.0324370403048241E-2</v>
+      </c>
+      <c r="G21" t="s">
+        <v>72</v>
+      </c>
+      <c r="H21" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I21" t="s">
+        <v>79</v>
+      </c>
+      <c r="J21" s="33">
+        <v>5.0324370403048241E-2</v>
+      </c>
+      <c r="L21" t="s">
+        <v>72</v>
+      </c>
+      <c r="M21" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N21" t="s">
+        <v>79</v>
+      </c>
+      <c r="O21" s="33">
+        <v>5.0324370403048241E-2</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>72</v>
+      </c>
+      <c r="R21" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S21" t="s">
+        <v>79</v>
+      </c>
+      <c r="T21" s="33">
+        <v>5.0324370403048241E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>72</v>
+      </c>
+      <c r="C22" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D22" t="s">
+        <v>80</v>
+      </c>
+      <c r="E22" s="33">
+        <v>4.644570688133022E-2</v>
+      </c>
+      <c r="G22" t="s">
+        <v>72</v>
+      </c>
+      <c r="H22" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I22" t="s">
+        <v>80</v>
+      </c>
+      <c r="J22" s="33">
+        <v>4.644570688133022E-2</v>
+      </c>
+      <c r="L22" t="s">
+        <v>72</v>
+      </c>
+      <c r="M22" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N22" t="s">
+        <v>80</v>
+      </c>
+      <c r="O22" s="33">
+        <v>4.644570688133022E-2</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>72</v>
+      </c>
+      <c r="R22" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S22" t="s">
+        <v>80</v>
+      </c>
+      <c r="T22" s="33">
+        <v>4.644570688133022E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
+        <v>72</v>
+      </c>
+      <c r="C23" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D23" t="s">
+        <v>81</v>
+      </c>
+      <c r="E23" s="35">
+        <v>3.198760977379362E-2</v>
+      </c>
+      <c r="G23" t="s">
+        <v>72</v>
+      </c>
+      <c r="H23" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I23" t="s">
+        <v>81</v>
+      </c>
+      <c r="J23" s="35">
+        <v>3.198760977379362E-2</v>
+      </c>
+      <c r="L23" t="s">
+        <v>72</v>
+      </c>
+      <c r="M23" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N23" t="s">
+        <v>81</v>
+      </c>
+      <c r="O23" s="35">
+        <v>3.198760977379362E-2</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>72</v>
+      </c>
+      <c r="R23" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S23" t="s">
+        <v>81</v>
+      </c>
+      <c r="T23" s="35">
+        <v>3.198760977379362E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
+        <v>72</v>
+      </c>
+      <c r="C24" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D24" t="s">
+        <v>82</v>
+      </c>
+      <c r="E24" s="35">
+        <v>3.450628688202826E-2</v>
+      </c>
+      <c r="G24" t="s">
+        <v>72</v>
+      </c>
+      <c r="H24" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I24" t="s">
+        <v>82</v>
+      </c>
+      <c r="J24" s="35">
+        <v>3.450628688202826E-2</v>
+      </c>
+      <c r="L24" t="s">
+        <v>72</v>
+      </c>
+      <c r="M24" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N24" t="s">
+        <v>82</v>
+      </c>
+      <c r="O24" s="35">
+        <v>3.450628688202826E-2</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>72</v>
+      </c>
+      <c r="R24" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S24" t="s">
+        <v>82</v>
+      </c>
+      <c r="T24" s="35">
+        <v>3.450628688202826E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B25" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D25" t="s">
+        <v>83</v>
+      </c>
+      <c r="E25" s="35">
+        <v>4.1710976210981882E-2</v>
+      </c>
+      <c r="G25" t="s">
+        <v>72</v>
+      </c>
+      <c r="H25" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I25" t="s">
+        <v>83</v>
+      </c>
+      <c r="J25" s="35">
+        <v>4.1710976210981882E-2</v>
+      </c>
+      <c r="L25" t="s">
+        <v>72</v>
+      </c>
+      <c r="M25" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N25" t="s">
+        <v>83</v>
+      </c>
+      <c r="O25" s="35">
+        <v>4.1710976210981882E-2</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>72</v>
+      </c>
+      <c r="R25" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S25" t="s">
+        <v>83</v>
+      </c>
+      <c r="T25" s="35">
+        <v>4.1710976210981882E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B26" t="s">
+        <v>72</v>
+      </c>
+      <c r="C26" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D26" t="s">
+        <v>84</v>
+      </c>
+      <c r="E26" s="35">
+        <v>4.110700091078253E-2</v>
+      </c>
+      <c r="G26" t="s">
+        <v>72</v>
+      </c>
+      <c r="H26" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I26" t="s">
+        <v>84</v>
+      </c>
+      <c r="J26" s="35">
+        <v>4.110700091078253E-2</v>
+      </c>
+      <c r="L26" t="s">
+        <v>72</v>
+      </c>
+      <c r="M26" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N26" t="s">
+        <v>84</v>
+      </c>
+      <c r="O26" s="35">
+        <v>4.110700091078253E-2</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>72</v>
+      </c>
+      <c r="R26" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S26" t="s">
+        <v>84</v>
+      </c>
+      <c r="T26" s="35">
+        <v>4.110700091078253E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B27" t="s">
+        <v>72</v>
+      </c>
+      <c r="C27" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D27" t="s">
+        <v>85</v>
+      </c>
+      <c r="E27" s="35">
+        <v>3.8350662386599552E-2</v>
+      </c>
+      <c r="G27" t="s">
+        <v>72</v>
+      </c>
+      <c r="H27" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I27" t="s">
+        <v>85</v>
+      </c>
+      <c r="J27" s="35">
+        <v>3.8350662386599552E-2</v>
+      </c>
+      <c r="L27" t="s">
+        <v>72</v>
+      </c>
+      <c r="M27" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N27" t="s">
+        <v>85</v>
+      </c>
+      <c r="O27" s="35">
+        <v>3.8350662386599552E-2</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>72</v>
+      </c>
+      <c r="R27" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S27" t="s">
+        <v>85</v>
+      </c>
+      <c r="T27" s="35">
+        <v>3.8350662386599552E-2</v>
+      </c>
+    </row>
+    <row r="28" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B28" t="s">
+        <v>72</v>
+      </c>
+      <c r="C28" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D28" t="s">
+        <v>86</v>
+      </c>
+      <c r="E28" s="35">
+        <v>3.7409762931132108E-2</v>
+      </c>
+      <c r="G28" t="s">
+        <v>72</v>
+      </c>
+      <c r="H28" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I28" t="s">
+        <v>86</v>
+      </c>
+      <c r="J28" s="35">
+        <v>3.7409762931132108E-2</v>
+      </c>
+      <c r="L28" t="s">
+        <v>72</v>
+      </c>
+      <c r="M28" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N28" t="s">
+        <v>86</v>
+      </c>
+      <c r="O28" s="35">
+        <v>3.7409762931132108E-2</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>72</v>
+      </c>
+      <c r="R28" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S28" t="s">
+        <v>86</v>
+      </c>
+      <c r="T28" s="35">
+        <v>3.7409762931132108E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B29" t="s">
+        <v>72</v>
+      </c>
+      <c r="C29" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D29" t="s">
+        <v>87</v>
+      </c>
+      <c r="E29" s="35">
+        <v>3.1132436657193206E-2</v>
+      </c>
+      <c r="G29" t="s">
+        <v>72</v>
+      </c>
+      <c r="H29" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I29" t="s">
+        <v>87</v>
+      </c>
+      <c r="J29" s="35">
+        <v>3.1132436657193206E-2</v>
+      </c>
+      <c r="L29" t="s">
+        <v>72</v>
+      </c>
+      <c r="M29" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N29" t="s">
+        <v>87</v>
+      </c>
+      <c r="O29" s="35">
+        <v>3.1132436657193206E-2</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>72</v>
+      </c>
+      <c r="R29" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S29" t="s">
+        <v>87</v>
+      </c>
+      <c r="T29" s="35">
+        <v>3.1132436657193206E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B30" t="s">
+        <v>72</v>
+      </c>
+      <c r="C30" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D30" t="s">
+        <v>88</v>
+      </c>
+      <c r="E30" s="35">
+        <v>3.3429633070020642E-2</v>
+      </c>
+      <c r="G30" t="s">
+        <v>72</v>
+      </c>
+      <c r="H30" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I30" t="s">
+        <v>88</v>
+      </c>
+      <c r="J30" s="35">
+        <v>3.3429633070020642E-2</v>
+      </c>
+      <c r="L30" t="s">
+        <v>72</v>
+      </c>
+      <c r="M30" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N30" t="s">
+        <v>88</v>
+      </c>
+      <c r="O30" s="35">
+        <v>3.3429633070020642E-2</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>72</v>
+      </c>
+      <c r="R30" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S30" t="s">
+        <v>88</v>
+      </c>
+      <c r="T30" s="35">
+        <v>3.3429633070020642E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B31" t="s">
+        <v>72</v>
+      </c>
+      <c r="C31" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D31" t="s">
+        <v>89</v>
+      </c>
+      <c r="E31" s="35">
+        <v>4.2259483749326171E-2</v>
+      </c>
+      <c r="G31" t="s">
+        <v>72</v>
+      </c>
+      <c r="H31" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I31" t="s">
+        <v>89</v>
+      </c>
+      <c r="J31" s="35">
+        <v>4.2259483749326171E-2</v>
+      </c>
+      <c r="L31" t="s">
+        <v>72</v>
+      </c>
+      <c r="M31" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N31" t="s">
+        <v>89</v>
+      </c>
+      <c r="O31" s="35">
+        <v>4.2259483749326171E-2</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>72</v>
+      </c>
+      <c r="R31" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S31" t="s">
+        <v>89</v>
+      </c>
+      <c r="T31" s="35">
+        <v>4.2259483749326171E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B32" t="s">
+        <v>72</v>
+      </c>
+      <c r="C32" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D32" t="s">
+        <v>90</v>
+      </c>
+      <c r="E32" s="35">
+        <v>4.1634467216423117E-2</v>
+      </c>
+      <c r="G32" t="s">
+        <v>72</v>
+      </c>
+      <c r="H32" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I32" t="s">
+        <v>90</v>
+      </c>
+      <c r="J32" s="35">
+        <v>4.1634467216423117E-2</v>
+      </c>
+      <c r="L32" t="s">
+        <v>72</v>
+      </c>
+      <c r="M32" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N32" t="s">
+        <v>90</v>
+      </c>
+      <c r="O32" s="35">
+        <v>4.1634467216423117E-2</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>72</v>
+      </c>
+      <c r="R32" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S32" t="s">
+        <v>90</v>
+      </c>
+      <c r="T32" s="35">
+        <v>4.1634467216423117E-2</v>
+      </c>
+    </row>
+    <row r="33" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B33" t="s">
+        <v>72</v>
+      </c>
+      <c r="C33" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D33" t="s">
+        <v>91</v>
+      </c>
+      <c r="E33" s="35">
+        <v>3.9259389280991014E-2</v>
+      </c>
+      <c r="G33" t="s">
+        <v>72</v>
+      </c>
+      <c r="H33" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I33" t="s">
+        <v>91</v>
+      </c>
+      <c r="J33" s="35">
+        <v>3.9259389280991014E-2</v>
+      </c>
+      <c r="L33" t="s">
+        <v>72</v>
+      </c>
+      <c r="M33" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N33" t="s">
+        <v>91</v>
+      </c>
+      <c r="O33" s="35">
+        <v>3.9259389280991014E-2</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>72</v>
+      </c>
+      <c r="R33" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S33" t="s">
+        <v>91</v>
+      </c>
+      <c r="T33" s="35">
+        <v>3.9259389280991014E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B34" t="s">
+        <v>72</v>
+      </c>
+      <c r="C34" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D34" t="s">
+        <v>92</v>
+      </c>
+      <c r="E34" s="35">
+        <v>3.742541478765557E-2</v>
+      </c>
+      <c r="G34" t="s">
+        <v>72</v>
+      </c>
+      <c r="H34" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I34" t="s">
+        <v>92</v>
+      </c>
+      <c r="J34" s="35">
+        <v>3.742541478765557E-2</v>
+      </c>
+      <c r="L34" t="s">
+        <v>72</v>
+      </c>
+      <c r="M34" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N34" t="s">
+        <v>92</v>
+      </c>
+      <c r="O34" s="35">
+        <v>3.742541478765557E-2</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>72</v>
+      </c>
+      <c r="R34" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S34" t="s">
+        <v>92</v>
+      </c>
+      <c r="T34" s="35">
+        <v>3.742541478765557E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B35" t="s">
+        <v>72</v>
+      </c>
+      <c r="C35" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D35" t="s">
+        <v>93</v>
+      </c>
+      <c r="E35" s="35">
+        <v>3.8818644082250733E-2</v>
+      </c>
+      <c r="G35" t="s">
+        <v>72</v>
+      </c>
+      <c r="H35" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I35" t="s">
+        <v>93</v>
+      </c>
+      <c r="J35" s="35">
+        <v>3.8818644082250733E-2</v>
+      </c>
+      <c r="L35" t="s">
+        <v>72</v>
+      </c>
+      <c r="M35" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N35" t="s">
+        <v>93</v>
+      </c>
+      <c r="O35" s="35">
+        <v>3.8818644082250733E-2</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>72</v>
+      </c>
+      <c r="R35" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S35" t="s">
+        <v>93</v>
+      </c>
+      <c r="T35" s="35">
+        <v>3.8818644082250733E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B36" t="s">
+        <v>72</v>
+      </c>
+      <c r="C36" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D36" t="s">
+        <v>94</v>
+      </c>
+      <c r="E36" s="35">
+        <v>4.101069729156176E-2</v>
+      </c>
+      <c r="G36" t="s">
+        <v>72</v>
+      </c>
+      <c r="H36" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I36" t="s">
+        <v>94</v>
+      </c>
+      <c r="J36" s="35">
+        <v>4.101069729156176E-2</v>
+      </c>
+      <c r="L36" t="s">
+        <v>72</v>
+      </c>
+      <c r="M36" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N36" t="s">
+        <v>94</v>
+      </c>
+      <c r="O36" s="35">
+        <v>4.101069729156176E-2</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>72</v>
+      </c>
+      <c r="R36" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S36" t="s">
+        <v>94</v>
+      </c>
+      <c r="T36" s="35">
+        <v>4.101069729156176E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B37" t="s">
+        <v>72</v>
+      </c>
+      <c r="C37" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D37" t="s">
+        <v>95</v>
+      </c>
+      <c r="E37" s="35">
+        <v>4.9652911424591967E-2</v>
+      </c>
+      <c r="G37" t="s">
+        <v>72</v>
+      </c>
+      <c r="H37" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I37" t="s">
+        <v>95</v>
+      </c>
+      <c r="J37" s="35">
+        <v>4.9652911424591967E-2</v>
+      </c>
+      <c r="L37" t="s">
+        <v>72</v>
+      </c>
+      <c r="M37" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N37" t="s">
+        <v>95</v>
+      </c>
+      <c r="O37" s="35">
+        <v>4.9652911424591967E-2</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>72</v>
+      </c>
+      <c r="R37" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S37" t="s">
+        <v>95</v>
+      </c>
+      <c r="T37" s="35">
+        <v>4.9652911424591967E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B38" t="s">
+        <v>72</v>
+      </c>
+      <c r="C38" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D38" t="s">
+        <v>96</v>
+      </c>
+      <c r="E38" s="35">
+        <v>4.9211095905815884E-2</v>
+      </c>
+      <c r="G38" t="s">
+        <v>72</v>
+      </c>
+      <c r="H38" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I38" t="s">
+        <v>96</v>
+      </c>
+      <c r="J38" s="35">
+        <v>4.9211095905815884E-2</v>
+      </c>
+      <c r="L38" t="s">
+        <v>72</v>
+      </c>
+      <c r="M38" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N38" t="s">
+        <v>96</v>
+      </c>
+      <c r="O38" s="35">
+        <v>4.9211095905815884E-2</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>72</v>
+      </c>
+      <c r="R38" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S38" t="s">
+        <v>96</v>
+      </c>
+      <c r="T38" s="35">
+        <v>4.9211095905815884E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B39" t="s">
+        <v>72</v>
+      </c>
+      <c r="C39" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D39" t="s">
+        <v>97</v>
+      </c>
+      <c r="E39" s="35">
+        <v>5.0243422728341029E-2</v>
+      </c>
+      <c r="G39" t="s">
+        <v>72</v>
+      </c>
+      <c r="H39" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I39" t="s">
+        <v>97</v>
+      </c>
+      <c r="J39" s="35">
+        <v>5.0243422728341029E-2</v>
+      </c>
+      <c r="L39" t="s">
+        <v>72</v>
+      </c>
+      <c r="M39" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N39" t="s">
+        <v>97</v>
+      </c>
+      <c r="O39" s="35">
+        <v>5.0243422728341029E-2</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>72</v>
+      </c>
+      <c r="R39" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S39" t="s">
+        <v>97</v>
+      </c>
+      <c r="T39" s="35">
+        <v>5.0243422728341029E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B40" t="s">
+        <v>72</v>
+      </c>
+      <c r="C40" t="str">
+        <f t="shared" si="0"/>
+        <v>DEMELC_COM</v>
+      </c>
+      <c r="D40" t="s">
+        <v>98</v>
+      </c>
+      <c r="E40" s="35">
+        <v>4.5311195975387637E-2</v>
+      </c>
+      <c r="G40" t="s">
+        <v>72</v>
+      </c>
+      <c r="H40" t="str">
+        <f t="shared" si="1"/>
+        <v>DEMELC_RSD</v>
+      </c>
+      <c r="I40" t="s">
+        <v>98</v>
+      </c>
+      <c r="J40" s="35">
+        <v>4.5311195975387637E-2</v>
+      </c>
+      <c r="L40" t="s">
+        <v>72</v>
+      </c>
+      <c r="M40" t="str">
+        <f t="shared" si="2"/>
+        <v>DEMELC_IND</v>
+      </c>
+      <c r="N40" t="s">
+        <v>98</v>
+      </c>
+      <c r="O40" s="35">
+        <v>4.5311195975387637E-2</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>72</v>
+      </c>
+      <c r="R40" t="str">
+        <f t="shared" si="3"/>
+        <v>DEMELC_TRA</v>
+      </c>
+      <c r="S40" t="s">
+        <v>98</v>
+      </c>
+      <c r="T40" s="35">
+        <v>4.5311195975387637E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>